<commit_message>
corrected folder sorting error in preprocessing whereby impossible and possible shapes were put in incorrect folder (yet to rerun cmats)
</commit_message>
<xml_diff>
--- a/Results/Study 1/Confusion Matrices (train images).xlsx
+++ b/Results/Study 1/Confusion Matrices (train images).xlsx
@@ -610,21 +610,21 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>527</v>
-      </c>
-      <c r="C2">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>118</v>
-      </c>
-      <c r="C3">
-        <v>522</v>
+        <v>537</v>
+      </c>
+      <c r="C2">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>125</v>
+      </c>
+      <c r="C3">
+        <v>515</v>
       </c>
     </row>
   </sheetData>
@@ -650,21 +650,21 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>508</v>
-      </c>
-      <c r="C2">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>213</v>
-      </c>
-      <c r="C3">
-        <v>427</v>
+        <v>495</v>
+      </c>
+      <c r="C2">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>218</v>
+      </c>
+      <c r="C3">
+        <v>422</v>
       </c>
     </row>
   </sheetData>

</xml_diff>